<commit_message>
corpus: Excel-written .xls of the add-in fixtures (#890)
Excel's SaveAs .xls of a workbook with an external link stops on the
Compatibility Checker even with CheckCompatibility and DisplayAlerts off.
The fixture script now presses its Continue button through UI Automation
from a background job, so addin-udf.xls and ext-name.xls are written by
Excel with no manual step. The .xlsx/.xlsb were regenerated in the same
run; they differ only in GUIDs, window position and the clone's path.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/legacy/addin/addin-udf.xlsx
+++ b/corpus/legacy/addin/addin-udf.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boris\source\workbench\docxy-issue-888\corpus\legacy\addin\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boris\source\workbench\docxy-issue-890\corpus\legacy\addin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD51738C-1224-4A84-8F73-FD5C09C514EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D75A86EC-BB10-4B52-96FD-F4FB88203886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{ECAE5278-FA83-41A2-9325-3EED8D57311C}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{37204B45-7399-42F2-9B6E-AB10A5E2F122}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -469,7 +469,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5C12CAB-F8E9-438F-A81B-A08B98E9BB8D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C869EB-7AC9-4059-A3F6-9E9B8A6BB5D3}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>